<commit_message>
Installing EF, creating new model, creating repo and services
</commit_message>
<xml_diff>
--- a/src/MesTâches.xlsx
+++ b/src/MesTâches.xlsx
@@ -23,6 +23,15 @@
   </x:si>
   <x:si>
     <x:t>Ma deuxième tâche</x:t>
+  </x:si>
+  <x:si>
+    <x:t>System.Windows.Controls.ComboBoxItem : À faire</x:t>
+  </x:si>
+  <x:si>
+    <x:t>System.Windows.Controls.ComboBoxItem : En cours</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Tâche 00001</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -391,24 +400,69 @@
   <x:dimension ref="A1:A2"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:1">
+    <x:row r="1" spans="1:3">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:1">
+    <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:1">
+    <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:1">
+    <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
         <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:3">
+      <x:c r="A5" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:3">
+      <x:c r="C7" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:3">
+      <x:c r="A8" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:3">
+      <x:c r="C10" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:3">
+      <x:c r="A11" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:3">
+      <x:c r="C13" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:3">
+      <x:c r="A14" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:3">
+      <x:c r="B15" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:3">
+      <x:c r="C16" s="0" t="s">
+        <x:v>5</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>